<commit_message>
KPI_Historico_Areas: append corte 2026_09
</commit_message>
<xml_diff>
--- a/Tablas/KPI_Historico_Areas.xlsx
+++ b/Tablas/KPI_Historico_Areas.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="81">
   <si>
     <t>Mes</t>
   </si>
@@ -251,6 +251,12 @@
   </si>
   <si>
     <t>PDF Analisis Monitor Gestión 2026 08 pag 20</t>
+  </si>
+  <si>
+    <t>tablero.yaml 2026_09 (analizar) [total]</t>
+  </si>
+  <si>
+    <t>tablero.yaml 2026_09 (analizar)</t>
   </si>
 </sst>
 </file>
@@ -586,7 +592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:14">
@@ -3236,6 +3242,358 @@
         <v>78</v>
       </c>
     </row>
+    <row r="66" spans="1:14">
+      <c r="A66" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B66">
+        <v>0</v>
+      </c>
+      <c r="C66" t="s">
+        <v>14</v>
+      </c>
+      <c r="D66">
+        <v>4073</v>
+      </c>
+      <c r="E66">
+        <v>0.15</v>
+      </c>
+      <c r="F66">
+        <v>0.72</v>
+      </c>
+      <c r="G66">
+        <v>0.55</v>
+      </c>
+      <c r="H66">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I66">
+        <v>0.6725</v>
+      </c>
+      <c r="J66">
+        <v>0.226</v>
+      </c>
+      <c r="K66">
+        <v>4</v>
+      </c>
+      <c r="L66">
+        <v>0.02</v>
+      </c>
+      <c r="M66">
+        <v>0.017</v>
+      </c>
+      <c r="N66" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14">
+      <c r="A67" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B67">
+        <v>3</v>
+      </c>
+      <c r="C67" t="s">
+        <v>15</v>
+      </c>
+      <c r="D67">
+        <v>468</v>
+      </c>
+      <c r="E67">
+        <v>-0.17</v>
+      </c>
+      <c r="F67">
+        <v>0.83</v>
+      </c>
+      <c r="G67">
+        <v>0.75</v>
+      </c>
+      <c r="H67">
+        <v>0.78</v>
+      </c>
+      <c r="I67">
+        <v>0.7915</v>
+      </c>
+      <c r="J67">
+        <v>0.295</v>
+      </c>
+      <c r="K67">
+        <v>3</v>
+      </c>
+      <c r="L67">
+        <v>0.01</v>
+      </c>
+      <c r="M67">
+        <v>0.023</v>
+      </c>
+      <c r="N67" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14">
+      <c r="A68" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B68">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>16</v>
+      </c>
+      <c r="D68">
+        <v>131</v>
+      </c>
+      <c r="E68">
+        <v>0.66</v>
+      </c>
+      <c r="F68">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="G68">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="H68">
+        <v>0.1</v>
+      </c>
+      <c r="I68">
+        <v>0.403</v>
+      </c>
+      <c r="J68">
+        <v>0.303</v>
+      </c>
+      <c r="K68">
+        <v>3</v>
+      </c>
+      <c r="L68">
+        <v>0.11</v>
+      </c>
+      <c r="M68">
+        <v>0</v>
+      </c>
+      <c r="N68" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14">
+      <c r="A69" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B69">
+        <v>6</v>
+      </c>
+      <c r="C69" t="s">
+        <v>17</v>
+      </c>
+      <c r="D69">
+        <v>470</v>
+      </c>
+      <c r="E69">
+        <v>0.21</v>
+      </c>
+      <c r="F69">
+        <v>0.15</v>
+      </c>
+      <c r="G69">
+        <v>0.28</v>
+      </c>
+      <c r="H69">
+        <v>0.57</v>
+      </c>
+      <c r="I69">
+        <v>0.365</v>
+      </c>
+      <c r="J69">
+        <v>0.323</v>
+      </c>
+      <c r="K69">
+        <v>10</v>
+      </c>
+      <c r="L69">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="M69">
+        <v>0.028</v>
+      </c>
+      <c r="N69" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14">
+      <c r="A70" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B70">
+        <v>7</v>
+      </c>
+      <c r="C70" t="s">
+        <v>18</v>
+      </c>
+      <c r="D70">
+        <v>95</v>
+      </c>
+      <c r="E70">
+        <v>-0.14</v>
+      </c>
+      <c r="F70">
+        <v>0.88</v>
+      </c>
+      <c r="G70">
+        <v>0.55</v>
+      </c>
+      <c r="H70">
+        <v>0.31</v>
+      </c>
+      <c r="I70">
+        <v>0.5575</v>
+      </c>
+      <c r="J70">
+        <v>0.31</v>
+      </c>
+      <c r="K70">
+        <v>3</v>
+      </c>
+      <c r="L70">
+        <v>0</v>
+      </c>
+      <c r="M70">
+        <v>0.048</v>
+      </c>
+      <c r="N70" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14">
+      <c r="A71" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B71">
+        <v>8</v>
+      </c>
+      <c r="C71" t="s">
+        <v>19</v>
+      </c>
+      <c r="D71">
+        <v>318</v>
+      </c>
+      <c r="E71">
+        <v>0.2</v>
+      </c>
+      <c r="F71">
+        <v>0.39</v>
+      </c>
+      <c r="G71">
+        <v>0.86</v>
+      </c>
+      <c r="H71">
+        <v>0.48</v>
+      </c>
+      <c r="I71">
+        <v>0.5245</v>
+      </c>
+      <c r="J71">
+        <v>0.203</v>
+      </c>
+      <c r="K71">
+        <v>2</v>
+      </c>
+      <c r="L71">
+        <v>0.02</v>
+      </c>
+      <c r="M71">
+        <v>0</v>
+      </c>
+      <c r="N71" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14">
+      <c r="A72" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B72">
+        <v>20</v>
+      </c>
+      <c r="C72" t="s">
+        <v>20</v>
+      </c>
+      <c r="D72">
+        <v>2076</v>
+      </c>
+      <c r="E72">
+        <v>0.24</v>
+      </c>
+      <c r="F72">
+        <v>0.88</v>
+      </c>
+      <c r="G72">
+        <v>0.47</v>
+      </c>
+      <c r="H72">
+        <v>0.73</v>
+      </c>
+      <c r="I72">
+        <v>0.7305</v>
+      </c>
+      <c r="J72">
+        <v>0.237</v>
+      </c>
+      <c r="K72">
+        <v>6</v>
+      </c>
+      <c r="L72">
+        <v>0.01</v>
+      </c>
+      <c r="M72">
+        <v>0.018</v>
+      </c>
+      <c r="N72" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14">
+      <c r="A73" s="1">
+        <v>46266</v>
+      </c>
+      <c r="B73">
+        <v>25</v>
+      </c>
+      <c r="C73" t="s">
+        <v>21</v>
+      </c>
+      <c r="D73">
+        <v>515</v>
+      </c>
+      <c r="E73">
+        <v>0.13</v>
+      </c>
+      <c r="F73">
+        <v>0.72</v>
+      </c>
+      <c r="G73">
+        <v>0.59</v>
+      </c>
+      <c r="H73">
+        <v>0.73</v>
+      </c>
+      <c r="I73">
+        <v>0.6985</v>
+      </c>
+      <c r="J73">
+        <v>0.056</v>
+      </c>
+      <c r="K73">
+        <v>4</v>
+      </c>
+      <c r="L73">
+        <v>0.03</v>
+      </c>
+      <c r="M73">
+        <v>0.008</v>
+      </c>
+      <c r="N73" t="s">
+        <v>80</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>